<commit_message>
Fix for Save Layout
</commit_message>
<xml_diff>
--- a/input/users.xlsx
+++ b/input/users.xlsx
@@ -397,7 +397,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:R8"/>
+  <dimension ref="A1:R3"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -407,7 +407,7 @@
         <v>username</v>
       </c>
       <c r="C1" t="str">
-        <v>passoword</v>
+        <v>password</v>
       </c>
       <c r="D1" t="str">
         <v>first_name</v>
@@ -457,22 +457,25 @@
     </row>
     <row r="2">
       <c r="A2">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="B2" t="str">
-        <v>BP001</v>
+        <v>BP006</v>
       </c>
       <c r="C2" t="str">
-        <v>System123#</v>
+        <v>System12345#</v>
       </c>
       <c r="D2" t="str">
-        <v>BP001</v>
+        <v>perf_test001</v>
+      </c>
+      <c r="E2" t="str">
+        <v>lastname_test001</v>
       </c>
       <c r="F2" t="str">
-        <v>BP001@newgensoft.com</v>
+        <v>agc_perf_test@test.com</v>
       </c>
       <c r="G2" t="str">
-        <v>CRI</v>
+        <v>CRI,CIV</v>
       </c>
       <c r="H2" t="str">
         <v>CRI#REGISTRY (CRI)</v>
@@ -490,42 +493,42 @@
         <v>Others</v>
       </c>
       <c r="M2" t="str">
-        <v>SPO</v>
+        <v>ADVOGRP(CRI)</v>
       </c>
       <c r="N2" t="str">
-        <v>ACL-05,AGCIW-4965</v>
+        <v>Crime Executives, CRI-ILCT, SVG</v>
       </c>
       <c r="O2" t="str">
-        <v>SKIP</v>
-      </c>
-      <c r="P2" t="str">
-        <v>Test Remarks</v>
+        <v>ADDUSERINGROUPROLE</v>
       </c>
       <c r="Q2" t="str">
-        <v>SKIPPED</v>
+        <v>SUCCESS</v>
       </c>
       <c r="R2" t="str">
-        <v>Action set to SKIP</v>
+        <v>Layout saved successfully using "View-Full" view</v>
       </c>
     </row>
     <row r="3">
       <c r="A3">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="B3" t="str">
-        <v>BP002</v>
+        <v>BP005</v>
       </c>
       <c r="C3" t="str">
-        <v>System123#</v>
+        <v>System12345#</v>
       </c>
       <c r="D3" t="str">
-        <v>BP002</v>
+        <v>perf_test001</v>
+      </c>
+      <c r="E3" t="str">
+        <v>lastname_test001</v>
       </c>
       <c r="F3" t="str">
-        <v>BP002@newgensoft.com</v>
+        <v>agc_perf_test@test.com</v>
       </c>
       <c r="G3" t="str">
-        <v>CRI</v>
+        <v>CRI,CIV</v>
       </c>
       <c r="H3" t="str">
         <v>CRI#REGISTRY (CRI)</v>
@@ -543,278 +546,29 @@
         <v>Others</v>
       </c>
       <c r="M3" t="str">
-        <v>ILCT</v>
+        <v>ADVOGRP(CRI)</v>
       </c>
       <c r="N3" t="str">
-        <v>ACL-05,AGCIW-4965</v>
+        <v>Crime Executives, CRI-ILCT, SVG</v>
       </c>
       <c r="O3" t="str">
-        <v>SKIP</v>
-      </c>
-      <c r="P3" t="str">
-        <v>Test Remarks</v>
+        <v>ADDUSERINGROUPROLE</v>
       </c>
       <c r="Q3" t="str">
-        <v>SKIPPED</v>
+        <v>SUCCESS</v>
       </c>
       <c r="R3" t="str">
-        <v>Action set to SKIP</v>
-      </c>
-    </row>
-    <row r="4">
-      <c r="A4">
-        <v>4</v>
-      </c>
-      <c r="B4" t="str">
-        <v>BP003</v>
-      </c>
-      <c r="C4" t="str">
-        <v>System123#</v>
-      </c>
-      <c r="D4" t="str">
-        <v>BP003</v>
-      </c>
-      <c r="F4" t="str">
-        <v>BP003@gmail.com</v>
-      </c>
-      <c r="G4" t="str">
-        <v>CRI</v>
-      </c>
-      <c r="H4" t="str">
-        <v>CRI#REGISTRY (CRI)</v>
-      </c>
-      <c r="I4" t="str">
-        <v>Singapore</v>
-      </c>
-      <c r="J4" t="str">
-        <v>No</v>
-      </c>
-      <c r="K4" t="str">
-        <v>CRI</v>
-      </c>
-      <c r="L4" t="str">
-        <v>Others</v>
-      </c>
-      <c r="M4" t="str">
-        <v>SPO</v>
-      </c>
-      <c r="N4" t="str">
-        <v>ACL-05,AGCIW-4965</v>
-      </c>
-      <c r="O4" t="str">
-        <v>SKIP</v>
-      </c>
-      <c r="P4" t="str">
-        <v>Test Remarks 3</v>
-      </c>
-      <c r="Q4" t="str">
-        <v>SKIPPED</v>
-      </c>
-      <c r="R4" t="str">
-        <v>Action set to SKIP</v>
-      </c>
-    </row>
-    <row r="5">
-      <c r="A5">
-        <v>5</v>
-      </c>
-      <c r="B5" t="str">
-        <v>BP004</v>
-      </c>
-      <c r="C5" t="str">
-        <v>System123#</v>
-      </c>
-      <c r="D5" t="str">
-        <v>BP004</v>
-      </c>
-      <c r="F5" t="str">
-        <v>BP004@gmail.com</v>
-      </c>
-      <c r="G5" t="str">
-        <v>CRI</v>
-      </c>
-      <c r="H5" t="str">
-        <v>CRI#REGISTRY (CRI)</v>
-      </c>
-      <c r="I5" t="str">
-        <v>Singapore</v>
-      </c>
-      <c r="J5" t="str">
-        <v>No</v>
-      </c>
-      <c r="K5" t="str">
-        <v>CRI</v>
-      </c>
-      <c r="L5" t="str">
-        <v>Others</v>
-      </c>
-      <c r="M5" t="str">
-        <v>ILCT</v>
-      </c>
-      <c r="N5" t="str">
-        <v>ACL-05,AGCIW-4965</v>
-      </c>
-      <c r="O5" t="str">
-        <v>SKIP</v>
-      </c>
-      <c r="P5" t="str">
-        <v>Test Remarks 4</v>
-      </c>
-      <c r="Q5" t="str">
-        <v>SKIPPED</v>
-      </c>
-      <c r="R5" t="str">
-        <v>Action set to SKIP</v>
-      </c>
-    </row>
-    <row r="6">
-      <c r="A6">
-        <v>6</v>
-      </c>
-      <c r="B6" t="str">
-        <v>BP005</v>
-      </c>
-      <c r="C6" t="str">
-        <v>System123#</v>
-      </c>
-      <c r="D6" t="str">
-        <v>BP005</v>
-      </c>
-      <c r="F6" t="str">
-        <v>BP005@gmail.com</v>
-      </c>
-      <c r="G6" t="str">
-        <v>CRI,CIV</v>
-      </c>
-      <c r="H6" t="str">
-        <v>CRI#REGISTRY (CRI)</v>
-      </c>
-      <c r="K6" t="str">
-        <v>CRI</v>
-      </c>
-      <c r="L6" t="str">
-        <v>Others</v>
-      </c>
-      <c r="O6" t="str">
-        <v>SKIP</v>
-      </c>
-      <c r="P6" t="str">
-        <v>Test Remarks 5</v>
-      </c>
-      <c r="Q6" t="str">
-        <v>SKIPPED</v>
-      </c>
-      <c r="R6" t="str">
-        <v>Action set to SKIP</v>
-      </c>
-    </row>
-    <row r="7">
-      <c r="A7">
-        <v>7</v>
-      </c>
-      <c r="B7" t="str">
-        <v>BP006</v>
-      </c>
-      <c r="C7" t="str">
-        <v>System123#</v>
-      </c>
-      <c r="D7" t="str">
-        <v>BP006</v>
-      </c>
-      <c r="F7" t="str">
-        <v>BP005@gmail.com</v>
-      </c>
-      <c r="G7" t="str">
-        <v>CRI</v>
-      </c>
-      <c r="H7" t="str">
-        <v>CRI#REGISTRY (CRI)</v>
-      </c>
-      <c r="K7" t="str">
-        <v>CRI</v>
-      </c>
-      <c r="L7" t="str">
-        <v>Others</v>
-      </c>
-      <c r="O7" t="str">
-        <v>SKIP</v>
-      </c>
-      <c r="P7" t="str">
-        <v>Test Remarks 6</v>
-      </c>
-      <c r="Q7" t="str">
-        <v>SKIPPED</v>
-      </c>
-      <c r="R7" t="str">
-        <v>Action set to SKIP</v>
-      </c>
-    </row>
-    <row r="8">
-      <c r="A8">
-        <v>98</v>
-      </c>
-      <c r="B8" t="str">
-        <v>BP007</v>
-      </c>
-      <c r="C8" t="str">
-        <v>System123#</v>
-      </c>
-      <c r="D8" t="str">
-        <v>BP007</v>
-      </c>
-      <c r="F8" t="str">
-        <v>BP001@newgensoft.com</v>
-      </c>
-      <c r="G8" t="str">
-        <v>CIV</v>
-      </c>
-      <c r="H8" t="str">
-        <v>CRI#REGISTRY (CRI)</v>
-      </c>
-      <c r="I8" t="str">
-        <v>Singapore</v>
-      </c>
-      <c r="J8" t="str">
-        <v>No</v>
-      </c>
-      <c r="K8" t="str">
-        <v>CRI</v>
-      </c>
-      <c r="L8" t="str">
-        <v>Others</v>
-      </c>
-      <c r="M8" t="str">
-        <v>ILCT</v>
-      </c>
-      <c r="N8" t="str">
-        <v>Litigation Group,AGCIW-4965,Group 1(CRI)</v>
-      </c>
-      <c r="O8" t="str">
-        <v>CREATE</v>
-      </c>
-      <c r="P8" t="str">
-        <v>Test Remarks 7</v>
-      </c>
-      <c r="Q8" t="str">
-        <v>SUCCESS</v>
-      </c>
-      <c r="R8" t="str">
-        <v>User created successfully</v>
+        <v>Layout saved successfully using "View-Full" view</v>
       </c>
     </row>
   </sheetData>
   <hyperlinks>
     <hyperlink ref="F2" r:id="rId1"/>
     <hyperlink ref="F3" r:id="rId2"/>
-    <hyperlink ref="F4" r:id="rId3"/>
-    <hyperlink ref="F5" r:id="rId4"/>
-    <hyperlink ref="F6" r:id="rId5"/>
-    <hyperlink ref="F7" r:id="rId6"/>
-    <hyperlink ref="F8" r:id="rId7"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:R8"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:R3"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>